<commit_message>
Checkpoint: Added a three-screen product teaser gallery, removed the hero gradient seam, linked FAQ removal requests to PhoennixAI, and strengthened the waitlist workbook with a local lifecycle test.
</commit_message>
<xml_diff>
--- a/kaizen-os-waitlist-system.xlsx
+++ b/kaizen-os-waitlist-system.xlsx
@@ -6,6 +6,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Waitlist" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field map" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Waitlist'!$A$1:$O$1001</definedName>
@@ -127,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -216,7 +217,7 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -234,8 +235,8 @@
     <xf numFmtId="166" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -253,6 +254,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -504,6 +508,36 @@
 </chartSpace>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Kaizen OS</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Unique key generated by the intake flow. Use this as the Key Column for every Excel Online update.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Use lowercase, trimmed email values. Duplicate addresses are blocked by the intake flow and highlighted here.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Timestamp for the waitlist submission, not product-account entry. Product entry is recorded in Joined date.</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <t>Audit timestamp written only when the person accepts the waitlist terms.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
@@ -537,8 +571,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WaitlistTable" displayName="WaitlistTable" ref="A1:O1001" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WaitlistTable" displayName="WaitlistTable" ref="A1:O1001" headerRowCount="1">
+  <autoFilter ref="A1:O1001"/>
+  <tableColumns count="15">
     <tableColumn id="1" name="Lead ID"/>
     <tableColumn id="2" name="First name"/>
     <tableColumn id="3" name="Email"/>
@@ -553,6 +588,7 @@
     <tableColumn id="12" name="Joined date"/>
     <tableColumn id="13" name="Source"/>
     <tableColumn id="14" name="Notes"/>
+    <tableColumn id="15" name="Terms accepted at"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -758,14 +794,14 @@
   <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="4" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -783,47 +819,36 @@
       <c r="H1" s="1" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="n"/>
-      <c r="B2" s="12" t="n"/>
-      <c r="C2" s="12" t="n"/>
-      <c r="D2" s="12" t="n"/>
-      <c r="E2" s="12" t="n"/>
-      <c r="F2" s="12" t="n"/>
-      <c r="G2" s="12" t="n"/>
-      <c r="H2" s="12" t="n"/>
+      <c r="A2" s="13" t="n"/>
+      <c r="B2" s="13" t="n"/>
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="13" t="n"/>
+      <c r="G2" s="13" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="43" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Demand</t>
         </is>
       </c>
-      <c r="B3" s="44" t="inlineStr">
+      <c r="B3" s="44" t="n"/>
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="43" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Pipeline</t>
         </is>
       </c>
-      <c r="C3" s="12" t="n"/>
-      <c r="D3" s="43" t="inlineStr">
-        <is>
-          <t>Pipeline status</t>
-        </is>
-      </c>
-      <c r="E3" s="45" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
+      <c r="E3" s="45" t="n"/>
+      <c r="F3" s="1" t="n"/>
       <c r="G3" s="43" t="inlineStr">
         <is>
           <t>Automation health</t>
         </is>
       </c>
-      <c r="H3" s="45" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
+      <c r="H3" s="45" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="46" t="inlineStr">
@@ -835,7 +860,7 @@
         <f>COUNTA(WaitlistTable[Email])</f>
         <v/>
       </c>
-      <c r="C4" s="12" t="n"/>
+      <c r="C4" s="13" t="n"/>
       <c r="D4" s="46" t="inlineStr">
         <is>
           <t>Waitlisted</t>
@@ -845,7 +870,7 @@
         <f>COUNTIF(WaitlistTable[Status],"Waitlisted")</f>
         <v/>
       </c>
-      <c r="F4" s="12" t="n"/>
+      <c r="F4" s="13" t="n"/>
       <c r="G4" s="48" t="inlineStr">
         <is>
           <t>Awaiting confirmation</t>
@@ -859,14 +884,14 @@
     <row r="5">
       <c r="A5" s="46" t="inlineStr">
         <is>
-          <t>Waitlisted</t>
+          <t>New in last 7 days</t>
         </is>
       </c>
       <c r="B5" s="47">
-        <f>COUNTIF(WaitlistTable[Status],"Waitlisted")</f>
+        <f>COUNTIFS(WaitlistTable[Joined at],"&gt;="&amp;TODAY()-7,WaitlistTable[Email],"&lt;&gt;")</f>
         <v/>
       </c>
-      <c r="C5" s="12" t="n"/>
+      <c r="C5" s="13" t="n"/>
       <c r="D5" s="46" t="inlineStr">
         <is>
           <t>Reviewing</t>
@@ -876,7 +901,7 @@
         <f>COUNTIF(WaitlistTable[Status],"Reviewing")</f>
         <v/>
       </c>
-      <c r="F5" s="12" t="n"/>
+      <c r="F5" s="13" t="n"/>
       <c r="G5" s="48" t="inlineStr">
         <is>
           <t>Ready to invite</t>
@@ -890,14 +915,14 @@
     <row r="6">
       <c r="A6" s="46" t="inlineStr">
         <is>
-          <t>Reviewing</t>
+          <t>Updates opt-ins</t>
         </is>
       </c>
       <c r="B6" s="47">
-        <f>COUNTIF(WaitlistTable[Status],"Reviewing")</f>
+        <f>COUNTIF(WaitlistTable[Updates opt-in],"Yes")</f>
         <v/>
       </c>
-      <c r="C6" s="12" t="n"/>
+      <c r="C6" s="13" t="n"/>
       <c r="D6" s="46" t="inlineStr">
         <is>
           <t>Invited</t>
@@ -907,7 +932,7 @@
         <f>COUNTIF(WaitlistTable[Status],"Invited")</f>
         <v/>
       </c>
-      <c r="F6" s="12" t="n"/>
+      <c r="F6" s="13" t="n"/>
       <c r="G6" s="48" t="inlineStr">
         <is>
           <t>Invitations sent</t>
@@ -921,14 +946,14 @@
     <row r="7">
       <c r="A7" s="46" t="inlineStr">
         <is>
-          <t>Invited</t>
+          <t>Confirmed signups</t>
         </is>
       </c>
       <c r="B7" s="47">
-        <f>COUNTIF(WaitlistTable[Status],"Invited")</f>
+        <f>COUNTIF(WaitlistTable[Confirmation sent],"Yes")</f>
         <v/>
       </c>
-      <c r="C7" s="12" t="n"/>
+      <c r="C7" s="13" t="n"/>
       <c r="D7" s="46" t="inlineStr">
         <is>
           <t>Joined</t>
@@ -938,10 +963,10 @@
         <f>COUNTIF(WaitlistTable[Status],"Joined")</f>
         <v/>
       </c>
-      <c r="F7" s="12" t="n"/>
+      <c r="F7" s="13" t="n"/>
       <c r="G7" s="48" t="inlineStr">
         <is>
-          <t>Conversion to joined</t>
+          <t>Join conversion</t>
         </is>
       </c>
       <c r="H7" s="49">
@@ -952,14 +977,14 @@
     <row r="8">
       <c r="A8" s="46" t="inlineStr">
         <is>
-          <t>Joined</t>
+          <t>Duplicate emails</t>
         </is>
       </c>
       <c r="B8" s="47">
-        <f>COUNTIF(WaitlistTable[Status],"Joined")</f>
+        <f>COUNTA(WaitlistTable[Email])-SUMPRODUCT((WaitlistTable[Email]&lt;&gt;"")/COUNTIF(WaitlistTable[Email],WaitlistTable[Email]&amp;""))</f>
         <v/>
       </c>
-      <c r="C8" s="12" t="n"/>
+      <c r="C8" s="13" t="n"/>
       <c r="D8" s="46" t="inlineStr">
         <is>
           <t>Declined</t>
@@ -969,100 +994,76 @@
         <f>COUNTIF(WaitlistTable[Status],"Declined")</f>
         <v/>
       </c>
-      <c r="F8" s="12" t="n"/>
+      <c r="F8" s="13" t="n"/>
       <c r="G8" s="48" t="n"/>
       <c r="H8" s="47" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="48" t="inlineStr">
+      <c r="A9" s="13" t="n"/>
+      <c r="B9" s="13" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="13" t="n"/>
+      <c r="F9" s="13" t="n"/>
+      <c r="G9" s="13" t="n"/>
+      <c r="H9" s="13" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="50" t="n"/>
+      <c r="B10" s="50" t="n"/>
+      <c r="C10" s="50" t="n"/>
+      <c r="D10" s="13" t="n"/>
+      <c r="E10" s="13" t="n"/>
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="13" t="n"/>
+      <c r="H10" s="13" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="51" t="inlineStr">
         <is>
-          <t>Declined</t>
+          <t>TEST-READY OPERATING ROUTINE</t>
         </is>
       </c>
-      <c r="B9" s="47">
-        <f>COUNTIF(WaitlistTable[Status],"Declined")</f>
-        <v/>
-      </c>
-      <c r="C9" s="12" t="n"/>
-      <c r="D9" s="48" t="n"/>
-      <c r="E9" s="47" t="n"/>
-      <c r="F9" s="12" t="n"/>
-      <c r="G9" s="48" t="n"/>
-      <c r="H9" s="47" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="50" t="inlineStr">
+      <c r="B11" s="1" t="n"/>
+      <c r="C11" s="1" t="n"/>
+      <c r="D11" s="1" t="n"/>
+      <c r="E11" s="1" t="n"/>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="n"/>
+      <c r="H11" s="1" t="n"/>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="52" t="inlineStr">
         <is>
-          <t>Invitation metric</t>
+          <t>1. Submit a non-production email through the website, then confirm one Waitlisted row and a Yes value for Confirmation sent.</t>
         </is>
       </c>
-      <c r="B10" s="47" t="inlineStr">
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="1" t="n"/>
+      <c r="D12" s="1" t="n"/>
+      <c r="E12" s="1" t="n"/>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="n"/>
+      <c r="H12" s="1" t="n"/>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="52" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>2. Submit the same address again. The intake flow must return a duplicate message and must not add a second row.</t>
         </is>
       </c>
-      <c r="C10" s="39" t="str"/>
-      <c r="D10" s="48" t="n"/>
-      <c r="E10" s="47" t="n"/>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="48" t="n"/>
-      <c r="H10" s="47" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="46" t="inlineStr">
+      <c r="B13" s="1" t="n"/>
+      <c r="C13" s="1" t="n"/>
+      <c r="D13" s="1" t="n"/>
+      <c r="E13" s="1" t="n"/>
+      <c r="F13" s="1" t="n"/>
+      <c r="G13" s="1" t="n"/>
+      <c r="H13" s="1" t="n"/>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="52" t="inlineStr">
         <is>
-          <t>Invitations sent</t>
-        </is>
-      </c>
-      <c r="B11" s="47">
-        <f>COUNTIF(Waitlist!$J$2:$J$201,"Yes")</f>
-        <v/>
-      </c>
-      <c r="C11" s="40" t="str"/>
-      <c r="D11" s="48" t="n"/>
-      <c r="E11" s="47" t="n"/>
-      <c r="F11" s="12" t="n"/>
-      <c r="G11" s="48" t="n"/>
-      <c r="H11" s="47" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="46" t="inlineStr">
-        <is>
-          <t>Updates opt-ins</t>
-        </is>
-      </c>
-      <c r="B12" s="46">
-        <f>COUNTIF(Waitlist!$H$2:$H$201,"Yes")</f>
-        <v/>
-      </c>
-      <c r="C12" s="40" t="str"/>
-      <c r="D12" s="48" t="n"/>
-      <c r="E12" s="48" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="48" t="n"/>
-      <c r="H12" s="48" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="40" t="inlineStr">
-        <is>
-          <t>Confirmed signups</t>
-        </is>
-      </c>
-      <c r="B13" s="40">
-        <f>COUNTIF(Waitlist!$I$2:$I$201,"Yes")</f>
-        <v/>
-      </c>
-      <c r="C13" s="40" t="str"/>
-      <c r="D13" s="12" t="n"/>
-      <c r="E13" s="12" t="n"/>
-      <c r="F13" s="12" t="n"/>
-      <c r="G13" s="12" t="n"/>
-      <c r="H13" s="12" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="51" t="inlineStr">
-        <is>
-          <t>Operating routine</t>
+          <t>3. Set the test record to Invited, run the scheduled invitation flow manually, and confirm Invitation sent plus Invitation date.</t>
         </is>
       </c>
       <c r="B14" s="1" t="n"/>
@@ -1073,10 +1074,10 @@
       <c r="G14" s="1" t="n"/>
       <c r="H14" s="1" t="n"/>
     </row>
-    <row r="15" ht="25" customHeight="1">
+    <row r="15" ht="28" customHeight="1">
       <c r="A15" s="52" t="inlineStr">
         <is>
-          <t>1. The intake flow adds a Waitlisted record and marks Confirmation sent after the Outlook email succeeds.</t>
+          <t>4. Call the joined flow from Kaizen OS, then confirm Status = Joined and a Joined date before clearing or declining the test row.</t>
         </is>
       </c>
       <c r="B15" s="1" t="n"/>
@@ -1087,176 +1088,164 @@
       <c r="G15" s="1" t="n"/>
       <c r="H15" s="1" t="n"/>
     </row>
-    <row r="16" ht="25" customHeight="1">
-      <c r="A16" s="52" t="inlineStr">
-        <is>
-          <t>2. Review new entries and set Status to Invited only when the person is ready for an invitation wave.</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="n"/>
-      <c r="C16" s="1" t="n"/>
-      <c r="D16" s="1" t="n"/>
-      <c r="E16" s="1" t="n"/>
-      <c r="F16" s="1" t="n"/>
-      <c r="G16" s="1" t="n"/>
-      <c r="H16" s="1" t="n"/>
-    </row>
-    <row r="17" ht="25" customHeight="1">
-      <c r="A17" s="52" t="inlineStr">
-        <is>
-          <t>3. The scheduled invitation flow sends people where Status = Invited and Invitation sent = No.</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="n"/>
-      <c r="C17" s="1" t="n"/>
-      <c r="D17" s="1" t="n"/>
-      <c r="E17" s="1" t="n"/>
-      <c r="F17" s="1" t="n"/>
-      <c r="G17" s="1" t="n"/>
-      <c r="H17" s="1" t="n"/>
-    </row>
-    <row r="18" ht="25" customHeight="1">
-      <c r="A18" s="52" t="inlineStr">
-        <is>
-          <t>4. Kaizen OS account creation should call the joined flow to set Status = Joined and record Joined date.</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="n"/>
-      <c r="C18" s="1" t="n"/>
-      <c r="D18" s="1" t="n"/>
-      <c r="E18" s="1" t="n"/>
-      <c r="F18" s="1" t="n"/>
-      <c r="G18" s="1" t="n"/>
-      <c r="H18" s="1" t="n"/>
+    <row r="16">
+      <c r="A16" s="13" t="n"/>
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="13" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="n"/>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="n"/>
+      <c r="D17" s="13" t="n"/>
+      <c r="E17" s="13" t="n"/>
+      <c r="F17" s="13" t="n"/>
+      <c r="G17" s="13" t="n"/>
+      <c r="H17" s="13" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="n"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="13" t="n"/>
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="13" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n"/>
-      <c r="B19" s="12" t="n"/>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="12" t="n"/>
-      <c r="E19" s="12" t="n"/>
-      <c r="F19" s="12" t="n"/>
-      <c r="G19" s="12" t="n"/>
-      <c r="H19" s="12" t="n"/>
+      <c r="A19" s="13" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="n"/>
+      <c r="E19" s="13" t="n"/>
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="13" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n"/>
-      <c r="B20" s="12" t="n"/>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="12" t="n"/>
-      <c r="F20" s="12" t="n"/>
-      <c r="G20" s="12" t="n"/>
-      <c r="H20" s="12" t="n"/>
+      <c r="A20" s="13" t="n"/>
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="13" t="n"/>
+      <c r="D20" s="13" t="n"/>
+      <c r="E20" s="13" t="n"/>
+      <c r="F20" s="13" t="n"/>
+      <c r="G20" s="13" t="n"/>
+      <c r="H20" s="13" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="n"/>
-      <c r="B21" s="12" t="n"/>
-      <c r="C21" s="12" t="n"/>
-      <c r="D21" s="12" t="n"/>
-      <c r="E21" s="12" t="n"/>
-      <c r="F21" s="12" t="n"/>
-      <c r="G21" s="12" t="n"/>
-      <c r="H21" s="12" t="n"/>
+      <c r="A21" s="13" t="n"/>
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="13" t="n"/>
+      <c r="D21" s="13" t="n"/>
+      <c r="E21" s="13" t="n"/>
+      <c r="F21" s="13" t="n"/>
+      <c r="G21" s="13" t="n"/>
+      <c r="H21" s="13" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="12" t="n"/>
-      <c r="F22" s="12" t="n"/>
-      <c r="G22" s="12" t="n"/>
-      <c r="H22" s="12" t="n"/>
+      <c r="A22" s="13" t="n"/>
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="n"/>
+      <c r="D22" s="13" t="n"/>
+      <c r="E22" s="13" t="n"/>
+      <c r="F22" s="13" t="n"/>
+      <c r="G22" s="13" t="n"/>
+      <c r="H22" s="13" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="n"/>
-      <c r="B23" s="12" t="n"/>
-      <c r="C23" s="12" t="n"/>
-      <c r="D23" s="12" t="n"/>
-      <c r="E23" s="12" t="n"/>
-      <c r="F23" s="12" t="n"/>
-      <c r="G23" s="12" t="n"/>
-      <c r="H23" s="12" t="n"/>
+      <c r="A23" s="13" t="n"/>
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="n"/>
+      <c r="D23" s="13" t="n"/>
+      <c r="E23" s="13" t="n"/>
+      <c r="F23" s="13" t="n"/>
+      <c r="G23" s="13" t="n"/>
+      <c r="H23" s="13" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n"/>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="12" t="n"/>
-      <c r="F24" s="12" t="n"/>
-      <c r="G24" s="12" t="n"/>
-      <c r="H24" s="12" t="n"/>
+      <c r="A24" s="13" t="n"/>
+      <c r="B24" s="13" t="n"/>
+      <c r="C24" s="13" t="n"/>
+      <c r="D24" s="13" t="n"/>
+      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="13" t="n"/>
+      <c r="G24" s="13" t="n"/>
+      <c r="H24" s="13" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n"/>
-      <c r="B25" s="12" t="n"/>
-      <c r="C25" s="12" t="n"/>
-      <c r="D25" s="12" t="n"/>
-      <c r="E25" s="12" t="n"/>
-      <c r="F25" s="12" t="n"/>
-      <c r="G25" s="12" t="n"/>
-      <c r="H25" s="12" t="n"/>
+      <c r="A25" s="13" t="n"/>
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="13" t="n"/>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="13" t="n"/>
+      <c r="F25" s="13" t="n"/>
+      <c r="G25" s="13" t="n"/>
+      <c r="H25" s="13" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n"/>
-      <c r="B26" s="12" t="n"/>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="12" t="n"/>
-      <c r="E26" s="12" t="n"/>
-      <c r="F26" s="12" t="n"/>
-      <c r="G26" s="12" t="n"/>
-      <c r="H26" s="12" t="n"/>
+      <c r="A26" s="13" t="n"/>
+      <c r="B26" s="13" t="n"/>
+      <c r="C26" s="13" t="n"/>
+      <c r="D26" s="13" t="n"/>
+      <c r="E26" s="13" t="n"/>
+      <c r="F26" s="13" t="n"/>
+      <c r="G26" s="13" t="n"/>
+      <c r="H26" s="13" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="n"/>
-      <c r="B27" s="12" t="n"/>
-      <c r="C27" s="12" t="n"/>
-      <c r="D27" s="12" t="n"/>
-      <c r="E27" s="12" t="n"/>
-      <c r="F27" s="12" t="n"/>
-      <c r="G27" s="12" t="n"/>
-      <c r="H27" s="12" t="n"/>
+      <c r="A27" s="13" t="n"/>
+      <c r="B27" s="13" t="n"/>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="13" t="n"/>
+      <c r="E27" s="13" t="n"/>
+      <c r="F27" s="13" t="n"/>
+      <c r="G27" s="13" t="n"/>
+      <c r="H27" s="13" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n"/>
-      <c r="B28" s="12" t="n"/>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="12" t="n"/>
-      <c r="E28" s="12" t="n"/>
-      <c r="F28" s="12" t="n"/>
-      <c r="G28" s="12" t="n"/>
-      <c r="H28" s="12" t="n"/>
+      <c r="A28" s="13" t="n"/>
+      <c r="B28" s="13" t="n"/>
+      <c r="C28" s="13" t="n"/>
+      <c r="D28" s="13" t="n"/>
+      <c r="E28" s="13" t="n"/>
+      <c r="F28" s="13" t="n"/>
+      <c r="G28" s="13" t="n"/>
+      <c r="H28" s="13" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="n"/>
-      <c r="B29" s="12" t="n"/>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="12" t="n"/>
-      <c r="E29" s="12" t="n"/>
-      <c r="F29" s="12" t="n"/>
-      <c r="G29" s="12" t="n"/>
-      <c r="H29" s="12" t="n"/>
+      <c r="A29" s="13" t="n"/>
+      <c r="B29" s="13" t="n"/>
+      <c r="C29" s="13" t="n"/>
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="13" t="n"/>
+      <c r="F29" s="13" t="n"/>
+      <c r="G29" s="13" t="n"/>
+      <c r="H29" s="13" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="n"/>
-      <c r="B30" s="12" t="n"/>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="12" t="n"/>
-      <c r="E30" s="12" t="n"/>
-      <c r="F30" s="12" t="n"/>
-      <c r="G30" s="12" t="n"/>
-      <c r="H30" s="12" t="n"/>
+      <c r="A30" s="13" t="n"/>
+      <c r="B30" s="13" t="n"/>
+      <c r="C30" s="13" t="n"/>
+      <c r="D30" s="13" t="n"/>
+      <c r="E30" s="13" t="n"/>
+      <c r="F30" s="13" t="n"/>
+      <c r="G30" s="13" t="n"/>
+      <c r="H30" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A12:H12"/>
     <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A11:H11"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1267,7 +1256,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:O1001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1277,7 +1266,7 @@
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -1289,7 +1278,7 @@
     <col width="22" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="53" t="inlineStr">
         <is>
           <t>Lead ID</t>
@@ -18398,15 +18387,20 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:I1001">
     <cfRule type="expression" priority="9" dxfId="4">
-      <formula>$I2="No"</formula>
+      <formula>AND($C2&lt;&gt;"",$I2="No")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J1001">
     <cfRule type="expression" priority="10" dxfId="4">
-      <formula>$J2="No"</formula>
+      <formula>AND($G2="Invited",$J2="No")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <conditionalFormatting sqref="C2:C1001">
+    <cfRule type="expression" priority="11" dxfId="7">
+      <formula>COUNTIF($C$2:$C$1001,$C2)&gt;1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="5">
     <dataValidation sqref="G2:G201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>Lists!$A$2:$A$6</formula1>
     </dataValidation>
@@ -18419,8 +18413,13 @@
     <dataValidation sqref="H2:J1001" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=Lists!$B$2:$B$3</formula1>
     </dataValidation>
+    <dataValidation sqref="C2:C1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Check email format" error="Enter a valid email address before saving this row." type="custom" errorStyle="stop">
+      <formula1>=OR(C2="",AND(ISNUMBER(SEARCH("@",C2)),ISNUMBER(SEARCH(".",C2))))</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
@@ -18500,4 +18499,295 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>Workbook field</t>
+        </is>
+      </c>
+      <c r="B1" s="57" t="inlineStr">
+        <is>
+          <t>Form / flow value</t>
+        </is>
+      </c>
+      <c r="C1" s="57" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="54" t="inlineStr">
+        <is>
+          <t>Lead ID</t>
+        </is>
+      </c>
+      <c r="B2" s="54" t="inlineStr">
+        <is>
+          <t>Generated in intake flow</t>
+        </is>
+      </c>
+      <c r="C2" s="54" t="inlineStr">
+        <is>
+          <t>Unique update key for Excel Online actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="54" t="inlineStr">
+        <is>
+          <t>First name</t>
+        </is>
+      </c>
+      <c r="B3" s="54" t="inlineStr">
+        <is>
+          <t>firstName</t>
+        </is>
+      </c>
+      <c r="C3" s="54" t="inlineStr">
+        <is>
+          <t>Required visitor name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="54" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="B4" s="54" t="inlineStr">
+        <is>
+          <t>Normalised email</t>
+        </is>
+      </c>
+      <c r="C4" s="54" t="inlineStr">
+        <is>
+          <t>Unique visitor identity; duplicate protected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="54" t="inlineStr">
+        <is>
+          <t>Company / Organisation</t>
+        </is>
+      </c>
+      <c r="B5" s="54" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="C5" s="54" t="inlineStr">
+        <is>
+          <t>Optional organisation context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="54" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B6" s="54" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>Optional role context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="54" t="inlineStr">
+        <is>
+          <t>Joined at</t>
+        </is>
+      </c>
+      <c r="B7" s="54" t="inlineStr">
+        <is>
+          <t>utcNow() at intake</t>
+        </is>
+      </c>
+      <c r="C7" s="54" t="inlineStr">
+        <is>
+          <t>When the person joined the waitlist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="54" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B8" s="54" t="inlineStr">
+        <is>
+          <t>Waitlisted / operator updates</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t>Lifecycle state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="54" t="inlineStr">
+        <is>
+          <t>Updates opt-in</t>
+        </is>
+      </c>
+      <c r="B9" s="54" t="inlineStr">
+        <is>
+          <t>updatesOptIn</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>Optional product-news consent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="54" t="inlineStr">
+        <is>
+          <t>Confirmation sent</t>
+        </is>
+      </c>
+      <c r="B10" s="54" t="inlineStr">
+        <is>
+          <t>Yes after Outlook success</t>
+        </is>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>Confirmation email state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="54" t="inlineStr">
+        <is>
+          <t>Invitation sent</t>
+        </is>
+      </c>
+      <c r="B11" s="54" t="inlineStr">
+        <is>
+          <t>Yes after scheduled flow</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>Invitation deduplication control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="54" t="inlineStr">
+        <is>
+          <t>Invitation date</t>
+        </is>
+      </c>
+      <c r="B12" s="54" t="inlineStr">
+        <is>
+          <t>utcNow() after invite</t>
+        </is>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>Invitation audit timestamp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="54" t="inlineStr">
+        <is>
+          <t>Joined date</t>
+        </is>
+      </c>
+      <c r="B13" s="54" t="inlineStr">
+        <is>
+          <t>utcNow() from joined flow</t>
+        </is>
+      </c>
+      <c r="C13" s="54" t="inlineStr">
+        <is>
+          <t>Product-account entry timestamp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="54" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B14" s="54" t="inlineStr">
+        <is>
+          <t>Kaizen OS waitlist website</t>
+        </is>
+      </c>
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t>Acquisition attribution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="54" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B15" s="54" t="inlineStr">
+        <is>
+          <t>Operator-only</t>
+        </is>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t>Internal review notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="54" t="inlineStr">
+        <is>
+          <t>Terms accepted at</t>
+        </is>
+      </c>
+      <c r="B16" s="54" t="inlineStr">
+        <is>
+          <t>utcNow() when termsAccepted</t>
+        </is>
+      </c>
+      <c r="C16" s="54" t="inlineStr">
+        <is>
+          <t>Terms acceptance audit.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>